<commit_message>
price_bank v0.9.3: no source column lost (pump diff pressure, leftover specs, unheaded and extra columns)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VJyVH74gN1Yg71dajtXmaL
</commit_message>
<xml_diff>
--- a/price_bank/test/fixtures_private/Compressors_bank_test_messy.xlsx
+++ b/price_bank/test/fixtures_private/Compressors_bank_test_messy.xlsx
@@ -1062,7 +1062,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:AK16"/>
+  <dimension ref="A3:AL16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="3">
@@ -1260,6 +1260,11 @@
           <t>Include in Totals (Y/N)</t>
         </is>
       </c>
+      <c r="AL6" t="inlineStr">
+        <is>
+          <t>Site Altitude (m)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -1428,6 +1433,9 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="AL7" t="n">
+        <v>705</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -1593,6 +1601,9 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="AL8" t="n">
+        <v>706</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -1758,6 +1769,9 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AL9" t="n">
+        <v>707</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -1926,6 +1940,9 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="AL10" t="n">
+        <v>708</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -2094,6 +2111,9 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="AL11" t="n">
+        <v>709</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -2253,6 +2273,9 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AL12" t="n">
+        <v>710</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -2412,6 +2435,9 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AL13" t="n">
+        <v>711</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -2571,6 +2597,9 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AL14" t="n">
+        <v>712</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -2739,6 +2768,9 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AL15" t="n">
+        <v>713</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -2906,6 +2938,9 @@
         <is>
           <t>Y</t>
         </is>
+      </c>
+      <c r="AL16" t="n">
+        <v>714</v>
       </c>
     </row>
   </sheetData>

</xml_diff>